<commit_message>
Updated German and English wordlist
- German: two new words, corrected weightings
- English: corrected weightings
</commit_message>
<xml_diff>
--- a/word-list/English.xlsx
+++ b/word-list/English.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KDrive\Project\Keyboard\keyboard heaven - in work\KeyDual Github readme\Wordlist 2026-04-20 files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KDrive\Project\Keyboard\keyboard heaven - in work\KeyDual Github readme\word-list 2026-04-20\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6E07B07C-33E5-49BB-B660-049F12E3309D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762C5CAC-282F-47D7-9FE8-54DE2FCFAB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5649" yWindow="2049" windowWidth="24685" windowHeight="13054" xr2:uid="{8354B6E7-B3CE-4353-AE33-8CFFFC12BD22}"/>
+    <workbookView xWindow="19886" yWindow="4054" windowWidth="12188" windowHeight="11332" xr2:uid="{8354B6E7-B3CE-4353-AE33-8CFFFC12BD22}"/>
   </bookViews>
   <sheets>
     <sheet name="100-wordlist-English" sheetId="1" r:id="rId1"/>
@@ -1370,7 +1370,7 @@
         <v>17</v>
       </c>
       <c r="C16">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
@@ -1381,7 +1381,7 @@
         <v>18</v>
       </c>
       <c r="C17">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.4">
@@ -1436,7 +1436,7 @@
         <v>23</v>
       </c>
       <c r="C22">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.4">
@@ -1480,7 +1480,7 @@
         <v>27</v>
       </c>
       <c r="C26">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.4">
@@ -1678,7 +1678,7 @@
         <v>45</v>
       </c>
       <c r="C44">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.4">
@@ -1711,7 +1711,7 @@
         <v>48</v>
       </c>
       <c r="C47">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.4">
@@ -1744,7 +1744,7 @@
         <v>51</v>
       </c>
       <c r="C50">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.4">
@@ -1777,7 +1777,7 @@
         <v>54</v>
       </c>
       <c r="C53">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.4">
@@ -1810,7 +1810,7 @@
         <v>57</v>
       </c>
       <c r="C56">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.4">
@@ -1843,7 +1843,7 @@
         <v>60</v>
       </c>
       <c r="C59">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.4">
@@ -1876,7 +1876,7 @@
         <v>63</v>
       </c>
       <c r="C62">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.4">
@@ -1909,7 +1909,7 @@
         <v>66</v>
       </c>
       <c r="C65">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.4">
@@ -1975,7 +1975,7 @@
         <v>72</v>
       </c>
       <c r="C71">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.4">
@@ -2074,7 +2074,7 @@
         <v>81</v>
       </c>
       <c r="C80">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.4">
@@ -2107,7 +2107,7 @@
         <v>84</v>
       </c>
       <c r="C83">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.4">
@@ -2140,7 +2140,7 @@
         <v>87</v>
       </c>
       <c r="C86">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.4">
@@ -2206,7 +2206,7 @@
         <v>93</v>
       </c>
       <c r="C92">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
Refined English word list
improves corpus coverage with minor impact on word frequency
</commit_message>
<xml_diff>
--- a/word-list/English.xlsx
+++ b/word-list/English.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KDrive\Project\Keyboard\keyboard heaven - in work\KeyDual Github readme\word-list 2026-04-20\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\KDrive\Project\Keyboard\keyboard heaven - in work\KeyDuel Word list\Keyduel_englis200_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{762C5CAC-282F-47D7-9FE8-54DE2FCFAB0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{09FF0B54-D2AA-4DC0-9532-6E07E6AFBA25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19886" yWindow="4054" windowWidth="12188" windowHeight="11332" xr2:uid="{8354B6E7-B3CE-4353-AE33-8CFFFC12BD22}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{43E84576-76D0-4934-8F4A-D6DB8E2906BA}"/>
   </bookViews>
   <sheets>
-    <sheet name="100-wordlist-English" sheetId="1" r:id="rId1"/>
+    <sheet name="English" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -72,7 +72,7 @@
     <t>time</t>
   </si>
   <si>
-    <t>good</t>
+    <t>come</t>
   </si>
   <si>
     <t>world</t>
@@ -90,16 +90,16 @@
     <t>some</t>
   </si>
   <si>
-    <t>just</t>
-  </si>
-  <si>
-    <t>life</t>
+    <t>said</t>
+  </si>
+  <si>
+    <t>should</t>
   </si>
   <si>
     <t>making</t>
   </si>
   <si>
-    <t>new</t>
+    <t>better</t>
   </si>
   <si>
     <t>right</t>
@@ -120,7 +120,7 @@
     <t>which</t>
   </si>
   <si>
-    <t>seem</t>
+    <t>results</t>
   </si>
   <si>
     <t>only</t>
@@ -132,7 +132,7 @@
     <t>so</t>
   </si>
   <si>
-    <t>used</t>
+    <t>done</t>
   </si>
   <si>
     <t>would</t>
@@ -141,7 +141,7 @@
     <t>will</t>
   </si>
   <si>
-    <t>tell</t>
+    <t>others</t>
   </si>
   <si>
     <t>man</t>
@@ -153,7 +153,7 @@
     <t>about</t>
   </si>
   <si>
-    <t>looked</t>
+    <t>place</t>
   </si>
   <si>
     <t>but</t>
@@ -168,7 +168,7 @@
     <t>are</t>
   </si>
   <si>
-    <t>way</t>
+    <t>state</t>
   </si>
   <si>
     <t>wanted</t>
@@ -204,7 +204,7 @@
     <t>be</t>
   </si>
   <si>
-    <t>long</t>
+    <t>concern</t>
   </si>
   <si>
     <t>know</t>
@@ -234,7 +234,7 @@
     <t>other</t>
   </si>
   <si>
-    <t>feel</t>
+    <t>problem</t>
   </si>
   <si>
     <t>or</t>
@@ -1193,7 +1193,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D326EBD1-BB7D-492C-8575-E3B89F38BC39}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA01EE50-579E-49A6-BFE4-77D89EB90ADA}">
   <dimension ref="A1:C101"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
@@ -1425,7 +1425,7 @@
         <v>22</v>
       </c>
       <c r="C21">
-        <v>0.6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.4">
@@ -1568,7 +1568,7 @@
         <v>35</v>
       </c>
       <c r="C34">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.4">
@@ -1645,7 +1645,7 @@
         <v>42</v>
       </c>
       <c r="C41">
-        <v>0.3</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.4">
@@ -1700,7 +1700,7 @@
         <v>47</v>
       </c>
       <c r="C46">
-        <v>0.6</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.4">

</xml_diff>